<commit_message>
Modificaciones190226 nuevo campo en claus actuals
</commit_message>
<xml_diff>
--- a/data/claus.xlsx
+++ b/data/claus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\_Flask_Python\gepV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5395BA09-338B-4C6C-8DEB-601795DDC49C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA8309A2-77AC-42CD-BFB0-4EA067238A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{954C4DF0-A74D-403B-AE99-890BAE94F81F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="216">
   <si>
     <t>Entrada + Campanar</t>
   </si>
@@ -672,13 +672,25 @@
   </si>
   <si>
     <t>P Entrada Escola</t>
+  </si>
+  <si>
+    <t>Caixeta</t>
+  </si>
+  <si>
+    <t>Cadenat</t>
+  </si>
+  <si>
+    <t>TOTS</t>
+  </si>
+  <si>
+    <t>actuals</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -696,33 +708,62 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <name val="Calibri"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -740,30 +781,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFDDEBF7"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFDDEBF7"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -795,100 +836,147 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF9BC2E6"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF9BC2E6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF9BC2E6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF9BC2E6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF9BC2E6"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1218,7 +1306,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFF8D717-D5CA-4BD4-8971-DA09B0A4DE2A}">
-  <dimension ref="A1:D184"/>
+  <dimension ref="A1:E196"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
@@ -1226,7 +1314,7 @@
     <col min="3" max="3" width="8.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>194</v>
       </c>
@@ -1239,8 +1327,11 @@
       <c r="D1" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E1" s="32" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1253,400 +1344,487 @@
       <c r="D2" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="E2" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="C3" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="10">
+        <v>3</v>
+      </c>
+      <c r="E3" s="34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="10">
+      <c r="C4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="E4" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="C5" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="10">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="E5" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="10">
+      <c r="C6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="E6" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="6">
+      <c r="C7" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="10">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="E7" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="10">
+      <c r="C8" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="E8" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D9" s="6">
+      <c r="C9" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="10">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="E9" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="10">
+      <c r="C10" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="6">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="E10" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="6">
+      <c r="C11" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="10">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="E11" s="34">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="10">
+      <c r="C12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="E12" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D13" s="6">
+      <c r="C13" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" s="10">
         <v>13</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
+      <c r="E13" s="35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D14" s="10">
+      <c r="C14" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6">
         <v>14</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="E14" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D15" s="6">
+      <c r="C15" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="10">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="E15" s="34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D16" s="10">
+      <c r="C16" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="E16" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D17" s="6">
+      <c r="C17" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D17" s="10">
         <v>17</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="E17" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="10">
+      <c r="C18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6">
         <v>18</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+      <c r="E18" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D19" s="6">
+      <c r="C19" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" s="10">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="E19" s="34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D20" s="10">
+      <c r="C20" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+      <c r="E20" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D21" s="6">
+      <c r="C21" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="10">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="E21" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D22" s="10">
+      <c r="C22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="6">
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="E22" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D23" s="6">
+      <c r="C23" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D23" s="10">
         <v>23</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="E23" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D24" s="10">
+      <c r="C24" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" s="6">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="E24" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="6">
+      <c r="C25" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" s="10">
         <v>25</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+      <c r="E25" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D26" s="10">
+      <c r="C26" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D26" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
+      <c r="E26" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D27" s="6">
+      <c r="C27" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D27" s="10">
         <v>27</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
+      <c r="E27" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" s="10">
+      <c r="C28" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="7" t="s">
+      <c r="E28" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D29" s="6">
+      <c r="C29" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D29" s="10">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="s">
+      <c r="E29" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D30" s="10">
+      <c r="C30" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E30" s="36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
         <v>33</v>
       </c>
@@ -1659,8 +1837,11 @@
       <c r="D31" s="10">
         <v>32</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E31" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>34</v>
       </c>
@@ -1673,8 +1854,11 @@
       <c r="D32" s="6">
         <v>33</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E32" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
         <v>197</v>
       </c>
@@ -1687,8 +1871,11 @@
       <c r="D33" s="14">
         <v>34</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E33" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
         <v>197</v>
       </c>
@@ -1701,8 +1888,11 @@
       <c r="D34" s="14">
         <v>35</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E34" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
         <v>198</v>
       </c>
@@ -1715,8 +1905,11 @@
       <c r="D35" s="17">
         <v>36</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E35" s="39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>199</v>
       </c>
@@ -1729,8 +1922,11 @@
       <c r="D36" s="6">
         <v>37</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E36" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
         <v>36</v>
       </c>
@@ -1743,162 +1939,198 @@
       <c r="D37" s="10">
         <v>38</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="11" t="s">
+      <c r="E37" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
         <v>200</v>
       </c>
       <c r="B38" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="C38" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D38" s="10">
+      <c r="C38" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D38" s="6">
         <v>40</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="7" t="s">
+      <c r="E38" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C39" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D39" s="6">
+      <c r="C39" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D39" s="10">
         <v>41</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="11" t="s">
+      <c r="E39" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="B40" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D40" s="10">
+      <c r="C40" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D40" s="6">
         <v>42</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="7" t="s">
+      <c r="E40" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D41" s="6">
+      <c r="C41" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D41" s="10">
         <v>43</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="11" t="s">
+      <c r="E41" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="B42" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D42" s="10">
+      <c r="C42" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D42" s="6">
         <v>44</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="7" t="s">
+      <c r="E42" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C43" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D43" s="6">
+      <c r="C43" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D43" s="10">
         <v>45</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="11" t="s">
+      <c r="E43" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="B44" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C44" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D44" s="10">
+      <c r="C44" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D44" s="6">
         <v>46</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="7" t="s">
+      <c r="E44" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D45" s="6">
+      <c r="C45" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D45" s="10">
         <v>47</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="11" t="s">
+      <c r="E45" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="B46" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C46" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D46" s="10">
+      <c r="C46" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" s="6">
         <v>48</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="7" t="s">
+      <c r="E46" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C47" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D47" s="6">
+      <c r="C47" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D47" s="10">
         <v>49</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="11" t="s">
+      <c r="E47" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="B48" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C48" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D48" s="10">
+      <c r="C48" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D48" s="6">
         <v>50</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E48" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
         <v>49</v>
       </c>
@@ -1911,8 +2143,11 @@
       <c r="D49" s="10">
         <v>52</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E49" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>50</v>
       </c>
@@ -1925,8 +2160,11 @@
       <c r="D50" s="6">
         <v>53</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E50" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="11" t="s">
         <v>52</v>
       </c>
@@ -1939,8 +2177,11 @@
       <c r="D51" s="10">
         <v>54</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E51" s="37">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>53</v>
       </c>
@@ -1953,8 +2194,11 @@
       <c r="D52" s="6">
         <v>57</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E52" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="11" t="s">
         <v>55</v>
       </c>
@@ -1967,8 +2211,11 @@
       <c r="D53" s="10">
         <v>62</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E53" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
         <v>57</v>
       </c>
@@ -1981,8 +2228,11 @@
       <c r="D54" s="6">
         <v>63</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E54" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="18" t="s">
         <v>58</v>
       </c>
@@ -1995,8 +2245,11 @@
       <c r="D55" s="14">
         <v>64</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E55" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
         <v>59</v>
       </c>
@@ -2009,8 +2262,11 @@
       <c r="D56" s="6">
         <v>65</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E56" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>60</v>
       </c>
@@ -2023,8 +2279,11 @@
       <c r="D57" s="10">
         <v>66</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E57" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
         <v>61</v>
       </c>
@@ -2037,8 +2296,11 @@
       <c r="D58" s="6">
         <v>67</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E58" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="11" t="s">
         <v>202</v>
       </c>
@@ -2051,8 +2313,11 @@
       <c r="D59" s="10">
         <v>73</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E59" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="18" t="s">
         <v>62</v>
       </c>
@@ -2065,8 +2330,11 @@
       <c r="D60" s="14">
         <v>74</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E60" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="18" t="s">
         <v>63</v>
       </c>
@@ -2079,8 +2347,11 @@
       <c r="D61" s="14">
         <v>78</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E61" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A62" s="18" t="s">
         <v>203</v>
       </c>
@@ -2093,8 +2364,11 @@
       <c r="D62" s="14">
         <v>102</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E62" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="18" t="s">
         <v>203</v>
       </c>
@@ -2107,8 +2381,11 @@
       <c r="D63" s="14">
         <v>105</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E63" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="18" t="s">
         <v>144</v>
       </c>
@@ -2121,8 +2398,11 @@
       <c r="D64" s="14">
         <v>112</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E64" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A65" s="18" t="s">
         <v>66</v>
       </c>
@@ -2135,8 +2415,11 @@
       <c r="D65" s="14">
         <v>122</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E65" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A66" s="18" t="s">
         <v>204</v>
       </c>
@@ -2149,8 +2432,11 @@
       <c r="D66" s="14">
         <v>131</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E66" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="18" t="s">
         <v>211</v>
       </c>
@@ -2163,8 +2449,11 @@
       <c r="D67" s="14">
         <v>134</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E67" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="18" t="s">
         <v>68</v>
       </c>
@@ -2174,11 +2463,14 @@
       <c r="C68" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D68" s="14">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D68" s="23">
+        <v>139</v>
+      </c>
+      <c r="E68" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="18" t="s">
         <v>205</v>
       </c>
@@ -2188,11 +2480,14 @@
       <c r="C69" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D69" s="14">
+      <c r="D69" s="23">
         <v>138</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E69" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>42</v>
       </c>
@@ -2205,8 +2500,11 @@
       <c r="D70" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E70" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="8" t="s">
         <v>72</v>
       </c>
@@ -2219,8 +2517,11 @@
       <c r="D71" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E71" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>73</v>
       </c>
@@ -2233,8 +2534,11 @@
       <c r="D72" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E72" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="8" t="s">
         <v>74</v>
       </c>
@@ -2247,8 +2551,11 @@
       <c r="D73" s="10">
         <v>4</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E73" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>206</v>
       </c>
@@ -2261,8 +2568,11 @@
       <c r="D74" s="6">
         <v>5</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E74" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="8" t="s">
         <v>207</v>
       </c>
@@ -2275,8 +2585,11 @@
       <c r="D75" s="10">
         <v>6</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E75" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>75</v>
       </c>
@@ -2289,8 +2602,11 @@
       <c r="D76" s="6">
         <v>7</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E76" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="8" t="s">
         <v>76</v>
       </c>
@@ -2303,8 +2619,11 @@
       <c r="D77" s="10">
         <v>8</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E77" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>77</v>
       </c>
@@ -2317,8 +2636,11 @@
       <c r="D78" s="6">
         <v>9</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E78" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A79" s="8" t="s">
         <v>78</v>
       </c>
@@ -2331,8 +2653,11 @@
       <c r="D79" s="10">
         <v>10</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E79" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>79</v>
       </c>
@@ -2345,8 +2670,11 @@
       <c r="D80" s="6">
         <v>11</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E80" s="36">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A81" s="8" t="s">
         <v>80</v>
       </c>
@@ -2359,8 +2687,11 @@
       <c r="D81" s="10">
         <v>12</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E81" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>82</v>
       </c>
@@ -2373,8 +2704,11 @@
       <c r="D82" s="6">
         <v>13</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E82" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A83" s="8" t="s">
         <v>83</v>
       </c>
@@ -2387,8 +2721,11 @@
       <c r="D83" s="10">
         <v>14</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E83" s="37">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A84" s="7" t="s">
         <v>84</v>
       </c>
@@ -2401,8 +2738,11 @@
       <c r="D84" s="6">
         <v>15</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E84" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="11" t="s">
         <v>85</v>
       </c>
@@ -2415,8 +2755,11 @@
       <c r="D85" s="10">
         <v>16</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E85" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A86" s="7" t="s">
         <v>86</v>
       </c>
@@ -2429,8 +2772,11 @@
       <c r="D86" s="6">
         <v>17</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E86" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A87" s="11" t="s">
         <v>87</v>
       </c>
@@ -2443,8 +2789,11 @@
       <c r="D87" s="10">
         <v>18</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E87" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A88" s="7" t="s">
         <v>88</v>
       </c>
@@ -2457,246 +2806,300 @@
       <c r="D88" s="6">
         <v>19</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A89" s="7" t="s">
+      <c r="E88" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A89" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B89" s="5" t="s">
+      <c r="B89" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C89" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D89" s="6">
+      <c r="C89" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D89" s="10">
         <v>21</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A90" s="11" t="s">
+      <c r="E89" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A90" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B90" s="9" t="s">
+      <c r="B90" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C90" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D90" s="10">
+      <c r="C90" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D90" s="6">
         <v>22</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A91" s="7" t="s">
+      <c r="E90" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A91" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="B91" s="5" t="s">
+      <c r="B91" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C91" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D91" s="6">
+      <c r="C91" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D91" s="10">
         <v>23</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" s="11" t="s">
+      <c r="E91" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A92" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B92" s="9" t="s">
+      <c r="B92" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C92" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D92" s="10">
+      <c r="C92" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D92" s="6">
         <v>24</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="7" t="s">
+      <c r="E92" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A93" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="B93" s="5" t="s">
+      <c r="B93" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C93" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D93" s="6">
+      <c r="C93" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D93" s="10">
         <v>25</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A94" s="11" t="s">
+      <c r="E93" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A94" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B94" s="9" t="s">
+      <c r="B94" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C94" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D94" s="10">
+      <c r="C94" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D94" s="6">
         <v>26</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A95" s="7" t="s">
+      <c r="E94" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A95" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="B95" s="5" t="s">
+      <c r="B95" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C95" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D95" s="6">
+      <c r="C95" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D95" s="10">
         <v>27</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A96" s="11" t="s">
+      <c r="E95" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A96" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B96" s="9" t="s">
+      <c r="B96" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C96" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D96" s="10">
+      <c r="C96" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D96" s="6">
         <v>28</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A97" s="7" t="s">
+      <c r="E96" s="40">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A97" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="B97" s="5" t="s">
+      <c r="B97" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C97" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D97" s="6">
+      <c r="C97" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D97" s="10">
         <v>29</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A98" s="11" t="s">
+      <c r="E97" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A98" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B98" s="9" t="s">
+      <c r="B98" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C98" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D98" s="10">
+      <c r="C98" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D98" s="6">
         <v>30</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A99" s="4" t="s">
+      <c r="E98" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A99" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B99" s="5" t="s">
+      <c r="B99" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C99" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D99" s="6">
+      <c r="C99" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D99" s="10">
         <v>31</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A100" s="8" t="s">
+      <c r="E99" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B100" s="9" t="s">
+      <c r="B100" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C100" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D100" s="10">
+      <c r="C100" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D100" s="6">
         <v>32</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A101" s="7" t="s">
+      <c r="E100" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A101" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B101" s="5" t="s">
+      <c r="B101" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C101" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D101" s="6">
+      <c r="C101" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D101" s="10">
         <v>33</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A102" s="11" t="s">
+      <c r="E101" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A102" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B102" s="9" t="s">
+      <c r="B102" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C102" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D102" s="10">
+      <c r="C102" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D102" s="6">
         <v>34</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A103" s="7" t="s">
+      <c r="E102" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A103" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="B103" s="5" t="s">
+      <c r="B103" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C103" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D103" s="6">
+      <c r="C103" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D103" s="10">
         <v>35</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="11" t="s">
+      <c r="E103" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A104" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B104" s="9" t="s">
+      <c r="B104" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C104" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D104" s="10">
+      <c r="C104" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D104" s="6">
         <v>36</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" s="7" t="s">
+      <c r="E104" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A105" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="B105" s="5" t="s">
+      <c r="B105" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C105" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D105" s="6">
+      <c r="C105" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D105" s="10">
         <v>37</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E105" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A106" s="18" t="s">
         <v>208</v>
       </c>
@@ -2709,218 +3112,266 @@
       <c r="D106" s="14">
         <v>38</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A107" s="7" t="s">
+      <c r="E106" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A107" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="B107" s="5" t="s">
+      <c r="B107" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C107" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D107" s="6">
+      <c r="C107" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D107" s="10">
         <v>39</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A108" s="11" t="s">
+      <c r="E107" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A108" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B108" s="9" t="s">
+      <c r="B108" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C108" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D108" s="10">
+      <c r="C108" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D108" s="6">
         <v>40</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A109" s="7" t="s">
+      <c r="E108" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A109" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="B109" s="5" t="s">
+      <c r="B109" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C109" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D109" s="6">
+      <c r="C109" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D109" s="10">
         <v>41</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A110" s="11" t="s">
+      <c r="E109" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A110" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B110" s="9" t="s">
+      <c r="B110" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C110" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D110" s="10">
+      <c r="C110" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D110" s="6">
         <v>42</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A111" s="7" t="s">
+      <c r="E110" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A111" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="B111" s="5" t="s">
+      <c r="B111" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C111" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D111" s="6">
+      <c r="C111" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D111" s="10">
         <v>43</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A112" s="11" t="s">
+      <c r="E111" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A112" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B112" s="9" t="s">
+      <c r="B112" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C112" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D112" s="10">
+      <c r="C112" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D112" s="6">
         <v>44</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E112" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A113" s="7" t="s">
         <v>114</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C113" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D113" s="6">
+      <c r="C113" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D113" s="10">
         <v>45</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A114" s="11" t="s">
+      <c r="E113" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A114" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B114" s="9" t="s">
+      <c r="B114" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C114" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D114" s="10">
+      <c r="C114" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D114" s="6">
         <v>46</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E114" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A115" s="7" t="s">
         <v>116</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C115" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D115" s="6">
+      <c r="C115" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D115" s="10">
         <v>47</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A116" s="11" t="s">
+      <c r="E115" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A116" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B116" s="9" t="s">
+      <c r="B116" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C116" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D116" s="10">
+      <c r="C116" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D116" s="6">
         <v>48</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E116" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A117" s="7" t="s">
         <v>118</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C117" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D117" s="6">
+      <c r="C117" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D117" s="10">
         <v>49</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A118" s="11" t="s">
+      <c r="E117" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A118" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B118" s="9" t="s">
+      <c r="B118" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C118" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D118" s="10">
+      <c r="C118" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D118" s="6">
         <v>50</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E118" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A119" s="7" t="s">
         <v>120</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C119" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D119" s="6">
+      <c r="C119" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D119" s="10">
         <v>51</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A120" s="11" t="s">
+      <c r="E119" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A120" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B120" s="9" t="s">
+      <c r="B120" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C120" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D120" s="10">
+      <c r="C120" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D120" s="6">
         <v>52</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A121" s="7" t="s">
+      <c r="E120" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A121" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="B121" s="5" t="s">
+      <c r="B121" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C121" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D121" s="6">
+      <c r="C121" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D121" s="10">
         <v>53</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E121" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A122" s="7" t="s">
         <v>123</v>
       </c>
@@ -2933,8 +3384,11 @@
       <c r="D122" s="6">
         <v>55</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E122" s="36">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A123" s="11" t="s">
         <v>125</v>
       </c>
@@ -2947,8 +3401,11 @@
       <c r="D123" s="10">
         <v>56</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E123" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A124" s="7" t="s">
         <v>126</v>
       </c>
@@ -2961,8 +3418,11 @@
       <c r="D124" s="6">
         <v>57</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E124" s="36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A125" s="11" t="s">
         <v>127</v>
       </c>
@@ -2975,8 +3435,11 @@
       <c r="D125" s="10">
         <v>58</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E125" s="37">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A126" s="7" t="s">
         <v>128</v>
       </c>
@@ -2989,8 +3452,11 @@
       <c r="D126" s="6">
         <v>59</v>
       </c>
-    </row>
-    <row r="127" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E126" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A127" s="11" t="s">
         <v>129</v>
       </c>
@@ -3003,148 +3469,181 @@
       <c r="D127" s="10">
         <v>60</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A128" s="11" t="s">
+      <c r="E127" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A128" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B128" s="9" t="s">
+      <c r="B128" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C128" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D128" s="10">
+      <c r="C128" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D128" s="6">
         <v>62</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A129" s="7" t="s">
+      <c r="E128" s="36">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A129" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="B129" s="5" t="s">
+      <c r="B129" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="C129" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D129" s="6">
+      <c r="C129" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D129" s="10">
         <v>63</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A130" s="11" t="s">
+      <c r="E129" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A130" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B130" s="9" t="s">
+      <c r="B130" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C130" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D130" s="10">
+      <c r="C130" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D130" s="6">
         <v>64</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A131" s="7" t="s">
+      <c r="E130" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A131" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="B131" s="5" t="s">
+      <c r="B131" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="C131" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D131" s="6">
+      <c r="C131" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D131" s="10">
         <v>65</v>
       </c>
-    </row>
-    <row r="132" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A132" s="11" t="s">
+      <c r="E131" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A132" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B132" s="9" t="s">
+      <c r="B132" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C132" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D132" s="10">
+      <c r="C132" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D132" s="6">
         <v>66</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A133" s="7" t="s">
+      <c r="E132" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A133" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B133" s="5" t="s">
+      <c r="B133" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C133" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D133" s="6">
+      <c r="C133" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D133" s="10">
         <v>67</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A134" s="11" t="s">
+      <c r="E133" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A134" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="B134" s="9" t="s">
+      <c r="B134" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C134" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D134" s="10">
+      <c r="C134" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D134" s="6">
         <v>68</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A135" s="7" t="s">
+      <c r="E134" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A135" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="B135" s="5" t="s">
+      <c r="B135" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C135" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D135" s="6">
+      <c r="C135" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D135" s="10">
         <v>69</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A136" s="11" t="s">
+      <c r="E135" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A136" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="B136" s="9" t="s">
+      <c r="B136" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C136" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D136" s="10">
+      <c r="C136" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D136" s="6">
         <v>70</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A137" s="7" t="s">
+      <c r="E136" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A137" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="B137" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="C137" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D137" s="6">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C137" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D137" s="10">
+        <v>71</v>
+      </c>
+      <c r="E137" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A138" s="7" t="s">
         <v>145</v>
       </c>
@@ -3157,9 +3656,12 @@
       <c r="D138" s="6">
         <v>101</v>
       </c>
-    </row>
-    <row r="139" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A139" s="23" t="s">
+      <c r="E138" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A139" s="24" t="s">
         <v>142</v>
       </c>
       <c r="B139" s="19" t="s">
@@ -3171,9 +3673,12 @@
       <c r="D139" s="14">
         <v>104</v>
       </c>
-    </row>
-    <row r="140" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A140" s="23" t="s">
+      <c r="E139" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A140" s="24" t="s">
         <v>142</v>
       </c>
       <c r="B140" s="19" t="s">
@@ -3185,9 +3690,12 @@
       <c r="D140" s="14">
         <v>108</v>
       </c>
-    </row>
-    <row r="141" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A141" s="23" t="s">
+      <c r="E140" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A141" s="24" t="s">
         <v>64</v>
       </c>
       <c r="B141" s="19" t="s">
@@ -3199,9 +3707,12 @@
       <c r="D141" s="14">
         <v>111</v>
       </c>
-    </row>
-    <row r="142" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A142" s="23" t="s">
+      <c r="E141" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A142" s="24" t="s">
         <v>64</v>
       </c>
       <c r="B142" s="19" t="s">
@@ -3213,9 +3724,12 @@
       <c r="D142" s="14">
         <v>112</v>
       </c>
-    </row>
-    <row r="143" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A143" s="23" t="s">
+      <c r="E142" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A143" s="24" t="s">
         <v>64</v>
       </c>
       <c r="B143" s="19" t="s">
@@ -3227,9 +3741,12 @@
       <c r="D143" s="14">
         <v>113</v>
       </c>
-    </row>
-    <row r="144" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A144" s="24" t="s">
+      <c r="E143" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A144" s="25" t="s">
         <v>143</v>
       </c>
       <c r="B144" s="21" t="s">
@@ -3238,12 +3755,15 @@
       <c r="C144" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D144" s="25">
+      <c r="D144" s="26">
         <v>127</v>
       </c>
-    </row>
-    <row r="145" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A145" s="23" t="s">
+      <c r="E144" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A145" s="24" t="s">
         <v>143</v>
       </c>
       <c r="B145" s="19" t="s">
@@ -3255,9 +3775,12 @@
       <c r="D145" s="14">
         <v>128</v>
       </c>
-    </row>
-    <row r="146" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A146" s="23" t="s">
+      <c r="E145" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A146" s="24" t="s">
         <v>144</v>
       </c>
       <c r="B146" s="19" t="s">
@@ -3269,540 +3792,1259 @@
       <c r="D146" s="14">
         <v>133</v>
       </c>
-    </row>
-    <row r="147" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E146" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A147" s="4" t="s">
         <v>147</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C147" s="26" t="s">
+      <c r="C147" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D147" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D147" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E147" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A148" s="11" t="s">
         <v>150</v>
       </c>
       <c r="B148" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C148" s="27" t="s">
+      <c r="C148" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D148" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D148" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E148" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A149" s="7" t="s">
         <v>151</v>
       </c>
       <c r="B149" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C149" s="26" t="s">
+      <c r="C149" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D149" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D149" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E149" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A150" s="8" t="s">
         <v>152</v>
       </c>
       <c r="B150" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C150" s="27" t="s">
+      <c r="C150" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D150" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D150" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E150" s="34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A151" s="4" t="s">
         <v>153</v>
       </c>
       <c r="B151" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="C151" s="26" t="s">
+      <c r="C151" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D151" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D151" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E151" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A152" s="8" t="s">
         <v>155</v>
       </c>
       <c r="B152" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C152" s="27" t="s">
+      <c r="C152" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D152" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D152" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E152" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
         <v>156</v>
       </c>
       <c r="B153" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C153" s="26" t="s">
+      <c r="C153" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D153" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D153" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E153" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A154" s="8" t="s">
         <v>157</v>
       </c>
       <c r="B154" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="C154" s="27" t="s">
+      <c r="C154" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D154" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D154" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E154" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A155" s="7" t="s">
         <v>159</v>
       </c>
       <c r="B155" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C155" s="26" t="s">
+      <c r="C155" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D155" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D155" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E155" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A156" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B156" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C156" s="27" t="s">
+      <c r="C156" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D156" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D156" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E156" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A157" s="7" t="s">
         <v>161</v>
       </c>
       <c r="B157" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C157" s="26" t="s">
+      <c r="C157" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D157" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D157" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E157" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A158" s="8" t="s">
         <v>162</v>
       </c>
       <c r="B158" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C158" s="27" t="s">
+      <c r="C158" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D158" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D158" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E158" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A159" s="7" t="s">
         <v>163</v>
       </c>
       <c r="B159" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C159" s="26" t="s">
+      <c r="C159" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D159" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D159" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E159" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A160" s="11" t="s">
         <v>164</v>
       </c>
       <c r="B160" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C160" s="27" t="s">
+      <c r="C160" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D160" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D160" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E160" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A161" s="7" t="s">
         <v>165</v>
       </c>
       <c r="B161" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C161" s="26" t="s">
+      <c r="C161" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D161" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D161" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E161" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A162" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="B162" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C162" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="D162" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="E162" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A163" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="B162" s="9" t="s">
+      <c r="B163" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C162" s="27" t="s">
+      <c r="C163" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D162" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A163" s="4" t="s">
+      <c r="D163" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E163" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A164" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="B163" s="5" t="s">
+      <c r="B164" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C163" s="26" t="s">
+      <c r="C164" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D163" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A164" s="11" t="s">
+      <c r="D164" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E164" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A165" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B164" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C164" s="27" t="s">
+      <c r="B165" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C165" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D164" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A165" s="7" t="s">
+      <c r="D165" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E165" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A166" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="B165" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C165" s="26" t="s">
+      <c r="B166" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C166" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D165" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A166" s="8" t="s">
+      <c r="D166" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E166" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A167" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B166" s="9" t="s">
+      <c r="B167" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C166" s="27" t="s">
+      <c r="C167" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D166" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A167" s="7" t="s">
+      <c r="D167" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E167" s="41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A168" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="B167" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C167" s="26" t="s">
+      <c r="B168" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C168" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D167" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A168" s="11" t="s">
+      <c r="D168" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E168" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A169" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B168" s="9" t="s">
+      <c r="B169" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C168" s="27" t="s">
+      <c r="C169" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D168" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A169" s="7" t="s">
+      <c r="D169" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E169" s="36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A170" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="B169" s="5" t="s">
+      <c r="B170" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="C169" s="26" t="s">
+      <c r="C170" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D169" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A170" s="11" t="s">
+      <c r="D170" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E170" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A171" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B170" s="9" t="s">
+      <c r="B171" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C170" s="27" t="s">
+      <c r="C171" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D170" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A171" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="B171" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C171" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="D171" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D171" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E171" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A172" s="8" t="s">
         <v>178</v>
       </c>
       <c r="B172" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C172" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="D172" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E172" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A173" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B173" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C172" s="27" t="s">
+      <c r="C173" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D172" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A173" s="7" t="s">
+      <c r="D173" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E173" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A174" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="B173" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C173" s="26" t="s">
+      <c r="B174" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C174" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D173" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A174" s="11" t="s">
+      <c r="D174" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E174" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A175" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="B174" s="9" t="s">
+      <c r="B175" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C174" s="27" t="s">
+      <c r="C175" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D174" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A175" s="7" t="s">
+      <c r="D175" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E175" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A176" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="B175" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C175" s="26" t="s">
+      <c r="B176" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C176" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D175" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A176" s="8" t="s">
+      <c r="D176" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E176" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A177" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="B176" s="9" t="s">
+      <c r="B177" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C176" s="27" t="s">
+      <c r="C177" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D176" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A177" s="4" t="s">
+      <c r="D177" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E177" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A178" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="B177" s="5" t="s">
+      <c r="B178" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="C177" s="26" t="s">
+      <c r="C178" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D177" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A178" s="11" t="s">
-        <v>186</v>
-      </c>
-      <c r="B178" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="C178" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="D178" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D178" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E178" s="34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A179" s="7" t="s">
         <v>186</v>
       </c>
       <c r="B179" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C179" s="26" t="s">
+        <v>187</v>
+      </c>
+      <c r="C179" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D179" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D179" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E179" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A180" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="B180" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C180" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="D180" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E180" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A181" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="B180" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C180" s="27" t="s">
+      <c r="B181" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C181" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D180" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A181" s="7" t="s">
+      <c r="D181" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E181" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A182" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="B181" s="5" t="s">
+      <c r="B182" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="C181" s="26" t="s">
+      <c r="C182" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D181" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A182" s="11" t="s">
+      <c r="D182" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E182" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A183" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="B182" s="9" t="s">
+      <c r="B183" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C182" s="27" t="s">
+      <c r="C183" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D182" s="27" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A183" s="7" t="s">
+      <c r="D183" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E183" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A184" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="B183" s="5" t="s">
+      <c r="B184" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="C183" s="26" t="s">
+      <c r="C184" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="D183" s="26" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A184" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="B184" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C184" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="D184" s="27" t="s">
-        <v>3</v>
+      <c r="D184" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="E184" s="34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A185" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B185" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C185" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D185" s="6">
+        <v>24</v>
+      </c>
+      <c r="E185" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A186" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B186" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C186" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D186" s="10">
+        <v>26</v>
+      </c>
+      <c r="E186" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A187" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B187" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C187" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D187" s="6">
+        <v>9</v>
+      </c>
+      <c r="E187" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A188" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B188" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C188" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D188" s="10">
+        <v>7</v>
+      </c>
+      <c r="E188" s="37">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A189" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B189" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C189" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D189" s="6">
+        <v>8</v>
+      </c>
+      <c r="E189" s="36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A190" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B190" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C190" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D190" s="10">
+        <v>1</v>
+      </c>
+      <c r="E190" s="37">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A191" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B191" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C191" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D191" s="6">
+        <v>5</v>
+      </c>
+      <c r="E191" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A192" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B192" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C192" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D192" s="10">
+        <v>6</v>
+      </c>
+      <c r="E192" s="37">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A193" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B193" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C193" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D193" s="6">
+        <v>2</v>
+      </c>
+      <c r="E193" s="36">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A194" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="B194" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C194" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D194" s="30">
+        <v>33</v>
+      </c>
+      <c r="E194" s="37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A195" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B195" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C195" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D195" s="31">
+        <v>4</v>
+      </c>
+      <c r="E195" s="36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A196" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="B196" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="C196" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D196" s="30">
+        <v>8</v>
+      </c>
+      <c r="E196" s="37">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E69">
+    <cfRule type="dataBar" priority="17">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{B18D320A-3FE6-4B08-8A4C-F0DAE9721D7A}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E62:E65">
+    <cfRule type="dataBar" priority="14">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{30A442DE-4081-468C-8AC8-FD799F5C2129}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E66">
+    <cfRule type="dataBar" priority="16">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{B52913C5-E451-4528-BAAE-3683A09401F3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E67">
+    <cfRule type="dataBar" priority="15">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{6A0DF1F2-87B4-4FD3-B883-472AC07A0192}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E70:E146">
+    <cfRule type="dataBar" priority="12">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{43F4B857-0E9C-434B-88C9-7CDCBA411C54}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="13" operator="between">
+      <formula>0</formula>
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E147:E184">
+    <cfRule type="dataBar" priority="10">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{E9A56A65-1FAC-4B4E-8681-2D215D09C8BE}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="11" operator="between">
+      <formula>1</formula>
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E185:E192">
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{05B7B619-D746-4D51-82BC-2974DF1B4FFC}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E185:E196">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="between">
+      <formula>0</formula>
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E186">
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{4C4A2CB4-C6E1-4CB5-BD3D-DE79C2EEDC0D}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E187">
+    <cfRule type="dataBar" priority="6">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{82303ACA-3CAC-4AA0-81A5-90C325F4D9D1}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E188:E189">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{234E19CE-17DA-4858-912E-D7625288100F}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E190">
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{8E2987B0-475E-447B-BC3E-91F116CAFA7D}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E191">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{D7AC83D4-D082-4BCB-A0FE-492A0BC469F7}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E192">
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{CA6181E5-F3F3-47B9-99EE-F6B486EA128A}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E193">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{80CA634F-B89D-440E-8BE2-0960B7FB89F3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{B18D320A-3FE6-4B08-8A4C-F0DAE9721D7A}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E2:E69</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{30A442DE-4081-468C-8AC8-FD799F5C2129}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E62:E65</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{B52913C5-E451-4528-BAAE-3683A09401F3}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E66</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{6A0DF1F2-87B4-4FD3-B883-472AC07A0192}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E67</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{43F4B857-0E9C-434B-88C9-7CDCBA411C54}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E70:E146</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{E9A56A65-1FAC-4B4E-8681-2D215D09C8BE}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E147:E184</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{05B7B619-D746-4D51-82BC-2974DF1B4FFC}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E185:E192</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{4C4A2CB4-C6E1-4CB5-BD3D-DE79C2EEDC0D}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E186</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{82303ACA-3CAC-4AA0-81A5-90C325F4D9D1}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E187</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{234E19CE-17DA-4858-912E-D7625288100F}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E188:E189</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{8E2987B0-475E-447B-BC3E-91F116CAFA7D}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E190</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{D7AC83D4-D082-4BCB-A0FE-492A0BC469F7}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E191</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{CA6181E5-F3F3-47B9-99EE-F6B486EA128A}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E192</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{80CA634F-B89D-440E-8BE2-0960B7FB89F3}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E193</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>